<commit_message>
Adaptations made to rjn script1
Changes made to run the model from scratch (after adding the folder with inputs)
</commit_message>
<xml_diff>
--- a/1. MSR Creator/ControlFile_MSRCreator.xlsx
+++ b/1. MSR Creator/ControlFile_MSRCreator.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="24332"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="24334"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Carlos\Desktop\Model-Supply-Regions-MSR-Toolset\1. MSR Creator\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Carlos\Desktop\MSR\Model-Supply-Regions-MSR-Toolset\1. MSR Creator\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BFA20CB0-B688-4422-A204-B1640FCEB711}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CEE40662-20C0-4EBC-8957-71C3C1A644A3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="24240" windowHeight="13020" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="23880" yWindow="-6870" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Paths" sheetId="9" r:id="rId1"/>
@@ -35,6 +35,9 @@
         <xcalcf:feature name="microsoft.com:CNMTM"/>
         <xcalcf:feature name="microsoft.com:LET_WF"/>
       </xcalcf:calcFeatures>
+    </ext>
+    <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
+      <xlwcv:version setVersion="1"/>
     </ext>
   </extLst>
 </workbook>
@@ -589,12 +592,6 @@
     <t>Enter turbine nameplate capacity in exponential form (kW) e.g. enter 1.96e6 for 1.96MW</t>
   </si>
   <si>
-    <t>C:\Users\Carlos\Desktop\Model-Supply-Regions-MSR-Toolset\1. MSR Creator</t>
-  </si>
-  <si>
-    <t>C:\Users\Carlos\Desktop\Model-Supply-Regions-MSR-Toolset\countrynames.csv</t>
-  </si>
-  <si>
     <t>Pixels below this value will be disregarded. Value can be changed by code if iterative relaxer mode is on. Units: m/s (****initially 6, but changed to include more surface)</t>
   </si>
   <si>
@@ -608,6 +605,12 @@
   </si>
   <si>
     <t>solarpv</t>
+  </si>
+  <si>
+    <t>C:\Users\Carlos\Desktop\MSR\Model-Supply-Regions-MSR-Toolset\1. MSR Creator</t>
+  </si>
+  <si>
+    <t>C:\Users\Carlos\Desktop\MSR\Model-Supply-Regions-MSR-Toolset\countrynames.csv</t>
   </si>
 </sst>
 </file>
@@ -1037,7 +1040,7 @@
         <v>3</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>173</v>
+        <v>178</v>
       </c>
       <c r="C2" s="2" t="s">
         <v>4</v>
@@ -1070,7 +1073,7 @@
         <v>11</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>174</v>
+        <v>179</v>
       </c>
       <c r="C5" s="2" t="s">
         <v>12</v>
@@ -1123,7 +1126,7 @@
         <v>20</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>177</v>
+        <v>175</v>
       </c>
     </row>
     <row r="4" spans="1:3" ht="45" x14ac:dyDescent="0.25">
@@ -1134,7 +1137,7 @@
         <v>0</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>178</v>
+        <v>176</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.25">
@@ -1175,7 +1178,7 @@
         <v>23</v>
       </c>
       <c r="B8" s="3" t="s">
-        <v>179</v>
+        <v>177</v>
       </c>
       <c r="C8" s="2" t="s">
         <v>24</v>
@@ -2352,7 +2355,7 @@
         <v>4</v>
       </c>
       <c r="C6" s="4" t="s">
-        <v>175</v>
+        <v>173</v>
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.25">
@@ -2407,7 +2410,7 @@
         <v>30</v>
       </c>
       <c r="C11" s="4" t="s">
-        <v>176</v>
+        <v>174</v>
       </c>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
Config changes for script 1
After running the model for solar resources (PV) changes were made to run the code for wind resources. Log files have also been flagged in the gitignore file to avoid tracking them.
</commit_message>
<xml_diff>
--- a/1. MSR Creator/ControlFile_MSRCreator.xlsx
+++ b/1. MSR Creator/ControlFile_MSRCreator.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Carlos\Desktop\MSR\Model-Supply-Regions-MSR-Toolset\1. MSR Creator\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CEE40662-20C0-4EBC-8957-71C3C1A644A3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7F023BA0-03A8-4520-93A5-BA2B32C98289}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="23880" yWindow="-6870" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="23880" yWindow="-6870" windowWidth="29040" windowHeight="15720" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Paths" sheetId="9" r:id="rId1"/>
@@ -604,13 +604,13 @@
     <t>Options=[0-No, 1-Yes]. Relax resource thresholds for resource lagging countries (***initially 0, but changed due to the mountain regions of Bolivia)</t>
   </si>
   <si>
-    <t>solarpv</t>
-  </si>
-  <si>
     <t>C:\Users\Carlos\Desktop\MSR\Model-Supply-Regions-MSR-Toolset\1. MSR Creator</t>
   </si>
   <si>
     <t>C:\Users\Carlos\Desktop\MSR\Model-Supply-Regions-MSR-Toolset\countrynames.csv</t>
+  </si>
+  <si>
+    <t>wind</t>
   </si>
 </sst>
 </file>
@@ -1040,7 +1040,7 @@
         <v>3</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="C2" s="2" t="s">
         <v>4</v>
@@ -1073,7 +1073,7 @@
         <v>11</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="C5" s="2" t="s">
         <v>12</v>
@@ -1178,7 +1178,7 @@
         <v>23</v>
       </c>
       <c r="B8" s="3" t="s">
-        <v>177</v>
+        <v>179</v>
       </c>
       <c r="C8" s="2" t="s">
         <v>24</v>
@@ -2352,7 +2352,7 @@
         <v>122</v>
       </c>
       <c r="B6" s="6">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="C6" s="4" t="s">
         <v>173</v>
@@ -2363,7 +2363,7 @@
         <v>123</v>
       </c>
       <c r="B7" s="6">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="C7" s="4" t="s">
         <v>124</v>

</xml_diff>